<commit_message>
Basic paket teknik kapsamı tanımlandı, fiyat 3.000₺
- Basic: basit vitrin (header + hero + kartlar + iletişim footer), responsive
  garanti + hover, profesyonel tasarım/palet değil. Reklam Basic'te yok.
- Opsiyonel Basit Destek 500₺ (aylık/talep başı netleştirilecek).
- Excel'e "Basic Paket Kapsam" sheet'i eklendi, Teklif Hesaplayıcı güncellendi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SN9GZYtUwLEGBFGLWQ18Ck
</commit_message>
<xml_diff>
--- a/🏰 300-Projects/Web Tasarım Freelance/Satış Planı.xlsx
+++ b/🏰 300-Projects/Web Tasarım Freelance/Satış Planı.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Özet &amp; Strateji" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Fiyatlandırma" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Teklif Hesaplayıcı" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Müşteri Takip" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Teknik Notlar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Basic Paket Kapsam" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Müşteri Takip" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Teknik Notlar" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -116,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -155,6 +156,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -807,7 +814,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Standart tasarım, responsive, interaktif</t>
+          <t>Basit vitrin: header + tanıtım görseli + kartlar + iletişim footer. Responsive garanti, hover efektleri. Profesyonel tasarım/renk paleti değil.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -816,7 +823,7 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="6">
@@ -935,7 +942,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3) AYLIK ABONELİKLER (bağımsız — müşteri hiçbirini ya da hepsini seçebilir)</t>
+          <t>3) DESTEK &amp; ABONELİKLER (bağımsız — müşteri hiçbirini ya da hepsini seçebilir)</t>
         </is>
       </c>
     </row>
@@ -947,7 +954,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Basic (₺/ay)</t>
+          <t>Basic (₺)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -964,48 +971,74 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Bakım (içerik update + monitoring + QA)</t>
+          <t>Basit Destek — Basic paket (hata düzeltme, içerik &amp; görsel değişimi, iletişim güncelleme)</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>800</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>1800</v>
+        <v>500</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Premium Support 7/24 (danışmanlık + on-call)</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>1500</v>
+          <t>Bakım (içerik update + monitoring + QA)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>2500</v>
+        <v>1200</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>4000</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Reklam Yönetimi (Google/Meta Ads + rapor)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>1500</v>
+          <t>Premium Support 7/24 (danışmanlık + on-call)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C19" s="5" t="n">
         <v>2500</v>
       </c>
       <c r="D19" s="5" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Reklam Yönetimi (Google/Meta Ads + rapor) — Basic pakette YOK</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D20" s="7" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1112,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1173,7 +1206,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>0</v>
@@ -1390,11 +1423,11 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Bakım</t>
+          <t>Basit Destek — Basic paket</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>0</v>
@@ -1407,11 +1440,11 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Premium Support 7/24</t>
+          <t>Bakım (Standart/Premium)</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>0</v>
@@ -1424,11 +1457,11 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Reklam Yönetimi</t>
+          <t>Premium Support 7/24</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>0</v>
@@ -1441,11 +1474,11 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>E-Commerce aylık</t>
+          <t>Reklam Yönetimi (Basic pakette YOK)</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>0</v>
@@ -1456,13 +1489,30 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>E-Commerce aylık</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="C26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="12">
+        <f>B26*C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>AYLIK TOPLAM</t>
         </is>
       </c>
-      <c r="D26" s="15">
-        <f>SUM(D22:D25)</f>
+      <c r="D27" s="15">
+        <f>SUM(D22:D26)</f>
         <v/>
       </c>
     </row>
@@ -1475,6 +1525,323 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Basic Paket — Teknik Kapsam  |  3.000₺ anahtar teslim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>AMAÇ: Müşterinin işini tanıtan + iletişim bilgisi sunan basit vitrin. Ziyaretçiyi müşterinin kendisine yönlendirir. Profesyonel tasarım hedefi YOK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Bölüm / Özellik</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Kapsam</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Dahil mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sayfa yapısı</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Tek index sayfası. Ek sayfa yok.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>1 adet üst başlık / menü.</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tanıtım görseli (hero)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Header altında ana sayfayı sunan görsel tarzı blok. Profesyonel site tasarımı değil.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Kartlar</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Hero altında işi / hizmetleri tanıtan kart bloğu.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Footer / kapanış</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>En altta iletişim bilgileri (telefon, adres, sosyal). Yeterli.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Logo</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Basit logo yapımı.</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Mobil / tablet / masaüstü uyum — GARANTİ (Basic'te bile).</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Hover efektleri</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Kart ve buton hover geçişleri.</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Renk paleti</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Standart palet. Profesyonel olması şart değil.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Domain + canlıya alma</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Domain alımı ve yayına alma dahil.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Ek sayfa (Hakkımızda, Ürünler vb.)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Sayfa başı ayrı ücret.</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Reklam yönetimi</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Basic pakette sunulmaz.</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Profesyonel / özel tasarım, animasyon</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Standart / Premium paket.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>E-commerce / online satış</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Ayrı modül.</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>OPSİYONEL — Basit Destek: 500₺</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Kapsam: hata düzeltme, içerik &amp; görsel değiştirme, iletişim bilgisi güncelleme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>AÇIK SORU: 500₺ aylık mı, talep başı mı? Akif netleştirecek.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A3:C4"/>
+    <mergeCell ref="A24:C24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1541,7 +1908,7 @@
           <t>Not</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>Durum seçenekleri: Aday / Görüşüldü / Teklif verildi / Kapora alındı / Üretimde / Teslim / Abonelik</t>
         </is>
@@ -1755,7 +2122,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>